<commit_message>
demo: re-stage T-12 workbook with the existence-gated monthly revenue helper
The helper row the T-6 annualized check reads now gates gross-scheduled-rent presence on
COUNTIF existence rather than a per-month nonzero total, so the workbook's T-6 figure
agrees with the preview's $3,859,652 on a printed row that has a zero month.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-t12-analysis.xlsx
+++ b/public/downloads/underwriting-demo/sample-t12-analysis.xlsx
@@ -2436,51 +2436,51 @@
         </is>
       </c>
       <c r="C39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",C$6:C$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",C$6:C$37),SUMIF($B$6:$B$37,"Gross Potential Rent",C$6:C$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",C$6:C$37))+SUMIF($B$6:$B$37,"Vacancy",C$6:C$37)+SUMIF($B$6:$B$37,"Concessions",C$6:C$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",C$6:C$37)+SUMIF($B$6:$B$37,"Delinquency",C$6:C$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",C$6:C$37)+SUMIF($B$6:$B$37,"Other Income",C$6:C$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",C$6:C$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",C$6:C$37),SUMIF($B$6:$B$37,"Gross Potential Rent",C$6:C$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",C$6:C$37))+SUMIF($B$6:$B$37,"Vacancy",C$6:C$37)+SUMIF($B$6:$B$37,"Concessions",C$6:C$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",C$6:C$37)+SUMIF($B$6:$B$37,"Delinquency",C$6:C$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",C$6:C$37)+SUMIF($B$6:$B$37,"Other Income",C$6:C$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",C$6:C$37)</f>
         <v/>
       </c>
       <c r="D39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",D$6:D$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",D$6:D$37),SUMIF($B$6:$B$37,"Gross Potential Rent",D$6:D$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",D$6:D$37))+SUMIF($B$6:$B$37,"Vacancy",D$6:D$37)+SUMIF($B$6:$B$37,"Concessions",D$6:D$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",D$6:D$37)+SUMIF($B$6:$B$37,"Delinquency",D$6:D$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",D$6:D$37)+SUMIF($B$6:$B$37,"Other Income",D$6:D$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",D$6:D$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",D$6:D$37),SUMIF($B$6:$B$37,"Gross Potential Rent",D$6:D$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",D$6:D$37))+SUMIF($B$6:$B$37,"Vacancy",D$6:D$37)+SUMIF($B$6:$B$37,"Concessions",D$6:D$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",D$6:D$37)+SUMIF($B$6:$B$37,"Delinquency",D$6:D$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",D$6:D$37)+SUMIF($B$6:$B$37,"Other Income",D$6:D$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",D$6:D$37)</f>
         <v/>
       </c>
       <c r="E39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",E$6:E$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",E$6:E$37),SUMIF($B$6:$B$37,"Gross Potential Rent",E$6:E$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",E$6:E$37))+SUMIF($B$6:$B$37,"Vacancy",E$6:E$37)+SUMIF($B$6:$B$37,"Concessions",E$6:E$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",E$6:E$37)+SUMIF($B$6:$B$37,"Delinquency",E$6:E$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",E$6:E$37)+SUMIF($B$6:$B$37,"Other Income",E$6:E$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",E$6:E$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",E$6:E$37),SUMIF($B$6:$B$37,"Gross Potential Rent",E$6:E$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",E$6:E$37))+SUMIF($B$6:$B$37,"Vacancy",E$6:E$37)+SUMIF($B$6:$B$37,"Concessions",E$6:E$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",E$6:E$37)+SUMIF($B$6:$B$37,"Delinquency",E$6:E$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",E$6:E$37)+SUMIF($B$6:$B$37,"Other Income",E$6:E$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",E$6:E$37)</f>
         <v/>
       </c>
       <c r="F39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",F$6:F$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",F$6:F$37),SUMIF($B$6:$B$37,"Gross Potential Rent",F$6:F$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",F$6:F$37))+SUMIF($B$6:$B$37,"Vacancy",F$6:F$37)+SUMIF($B$6:$B$37,"Concessions",F$6:F$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",F$6:F$37)+SUMIF($B$6:$B$37,"Delinquency",F$6:F$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",F$6:F$37)+SUMIF($B$6:$B$37,"Other Income",F$6:F$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",F$6:F$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",F$6:F$37),SUMIF($B$6:$B$37,"Gross Potential Rent",F$6:F$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",F$6:F$37))+SUMIF($B$6:$B$37,"Vacancy",F$6:F$37)+SUMIF($B$6:$B$37,"Concessions",F$6:F$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",F$6:F$37)+SUMIF($B$6:$B$37,"Delinquency",F$6:F$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",F$6:F$37)+SUMIF($B$6:$B$37,"Other Income",F$6:F$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",F$6:F$37)</f>
         <v/>
       </c>
       <c r="G39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",G$6:G$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",G$6:G$37),SUMIF($B$6:$B$37,"Gross Potential Rent",G$6:G$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",G$6:G$37))+SUMIF($B$6:$B$37,"Vacancy",G$6:G$37)+SUMIF($B$6:$B$37,"Concessions",G$6:G$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",G$6:G$37)+SUMIF($B$6:$B$37,"Delinquency",G$6:G$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",G$6:G$37)+SUMIF($B$6:$B$37,"Other Income",G$6:G$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",G$6:G$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",G$6:G$37),SUMIF($B$6:$B$37,"Gross Potential Rent",G$6:G$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",G$6:G$37))+SUMIF($B$6:$B$37,"Vacancy",G$6:G$37)+SUMIF($B$6:$B$37,"Concessions",G$6:G$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",G$6:G$37)+SUMIF($B$6:$B$37,"Delinquency",G$6:G$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",G$6:G$37)+SUMIF($B$6:$B$37,"Other Income",G$6:G$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",G$6:G$37)</f>
         <v/>
       </c>
       <c r="H39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",H$6:H$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",H$6:H$37),SUMIF($B$6:$B$37,"Gross Potential Rent",H$6:H$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",H$6:H$37))+SUMIF($B$6:$B$37,"Vacancy",H$6:H$37)+SUMIF($B$6:$B$37,"Concessions",H$6:H$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",H$6:H$37)+SUMIF($B$6:$B$37,"Delinquency",H$6:H$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",H$6:H$37)+SUMIF($B$6:$B$37,"Other Income",H$6:H$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",H$6:H$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",H$6:H$37),SUMIF($B$6:$B$37,"Gross Potential Rent",H$6:H$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",H$6:H$37))+SUMIF($B$6:$B$37,"Vacancy",H$6:H$37)+SUMIF($B$6:$B$37,"Concessions",H$6:H$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",H$6:H$37)+SUMIF($B$6:$B$37,"Delinquency",H$6:H$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",H$6:H$37)+SUMIF($B$6:$B$37,"Other Income",H$6:H$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",H$6:H$37)</f>
         <v/>
       </c>
       <c r="I39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",I$6:I$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",I$6:I$37),SUMIF($B$6:$B$37,"Gross Potential Rent",I$6:I$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",I$6:I$37))+SUMIF($B$6:$B$37,"Vacancy",I$6:I$37)+SUMIF($B$6:$B$37,"Concessions",I$6:I$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",I$6:I$37)+SUMIF($B$6:$B$37,"Delinquency",I$6:I$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",I$6:I$37)+SUMIF($B$6:$B$37,"Other Income",I$6:I$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",I$6:I$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",I$6:I$37),SUMIF($B$6:$B$37,"Gross Potential Rent",I$6:I$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",I$6:I$37))+SUMIF($B$6:$B$37,"Vacancy",I$6:I$37)+SUMIF($B$6:$B$37,"Concessions",I$6:I$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",I$6:I$37)+SUMIF($B$6:$B$37,"Delinquency",I$6:I$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",I$6:I$37)+SUMIF($B$6:$B$37,"Other Income",I$6:I$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",I$6:I$37)</f>
         <v/>
       </c>
       <c r="J39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",J$6:J$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",J$6:J$37),SUMIF($B$6:$B$37,"Gross Potential Rent",J$6:J$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",J$6:J$37))+SUMIF($B$6:$B$37,"Vacancy",J$6:J$37)+SUMIF($B$6:$B$37,"Concessions",J$6:J$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",J$6:J$37)+SUMIF($B$6:$B$37,"Delinquency",J$6:J$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",J$6:J$37)+SUMIF($B$6:$B$37,"Other Income",J$6:J$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",J$6:J$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",J$6:J$37),SUMIF($B$6:$B$37,"Gross Potential Rent",J$6:J$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",J$6:J$37))+SUMIF($B$6:$B$37,"Vacancy",J$6:J$37)+SUMIF($B$6:$B$37,"Concessions",J$6:J$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",J$6:J$37)+SUMIF($B$6:$B$37,"Delinquency",J$6:J$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",J$6:J$37)+SUMIF($B$6:$B$37,"Other Income",J$6:J$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",J$6:J$37)</f>
         <v/>
       </c>
       <c r="K39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",K$6:K$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",K$6:K$37),SUMIF($B$6:$B$37,"Gross Potential Rent",K$6:K$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",K$6:K$37))+SUMIF($B$6:$B$37,"Vacancy",K$6:K$37)+SUMIF($B$6:$B$37,"Concessions",K$6:K$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",K$6:K$37)+SUMIF($B$6:$B$37,"Delinquency",K$6:K$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",K$6:K$37)+SUMIF($B$6:$B$37,"Other Income",K$6:K$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",K$6:K$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",K$6:K$37),SUMIF($B$6:$B$37,"Gross Potential Rent",K$6:K$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",K$6:K$37))+SUMIF($B$6:$B$37,"Vacancy",K$6:K$37)+SUMIF($B$6:$B$37,"Concessions",K$6:K$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",K$6:K$37)+SUMIF($B$6:$B$37,"Delinquency",K$6:K$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",K$6:K$37)+SUMIF($B$6:$B$37,"Other Income",K$6:K$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",K$6:K$37)</f>
         <v/>
       </c>
       <c r="L39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",L$6:L$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",L$6:L$37),SUMIF($B$6:$B$37,"Gross Potential Rent",L$6:L$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",L$6:L$37))+SUMIF($B$6:$B$37,"Vacancy",L$6:L$37)+SUMIF($B$6:$B$37,"Concessions",L$6:L$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",L$6:L$37)+SUMIF($B$6:$B$37,"Delinquency",L$6:L$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",L$6:L$37)+SUMIF($B$6:$B$37,"Other Income",L$6:L$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",L$6:L$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",L$6:L$37),SUMIF($B$6:$B$37,"Gross Potential Rent",L$6:L$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",L$6:L$37))+SUMIF($B$6:$B$37,"Vacancy",L$6:L$37)+SUMIF($B$6:$B$37,"Concessions",L$6:L$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",L$6:L$37)+SUMIF($B$6:$B$37,"Delinquency",L$6:L$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",L$6:L$37)+SUMIF($B$6:$B$37,"Other Income",L$6:L$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",L$6:L$37)</f>
         <v/>
       </c>
       <c r="M39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",M$6:M$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",M$6:M$37),SUMIF($B$6:$B$37,"Gross Potential Rent",M$6:M$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",M$6:M$37))+SUMIF($B$6:$B$37,"Vacancy",M$6:M$37)+SUMIF($B$6:$B$37,"Concessions",M$6:M$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",M$6:M$37)+SUMIF($B$6:$B$37,"Delinquency",M$6:M$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",M$6:M$37)+SUMIF($B$6:$B$37,"Other Income",M$6:M$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",M$6:M$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",M$6:M$37),SUMIF($B$6:$B$37,"Gross Potential Rent",M$6:M$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",M$6:M$37))+SUMIF($B$6:$B$37,"Vacancy",M$6:M$37)+SUMIF($B$6:$B$37,"Concessions",M$6:M$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",M$6:M$37)+SUMIF($B$6:$B$37,"Delinquency",M$6:M$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",M$6:M$37)+SUMIF($B$6:$B$37,"Other Income",M$6:M$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",M$6:M$37)</f>
         <v/>
       </c>
       <c r="N39" s="11">
-        <f>IF(SUMIF($B$6:$B$37,"Gross Scheduled Rent",N$6:N$37)&lt;&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",N$6:N$37),SUMIF($B$6:$B$37,"Gross Potential Rent",N$6:N$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",N$6:N$37))+SUMIF($B$6:$B$37,"Vacancy",N$6:N$37)+SUMIF($B$6:$B$37,"Concessions",N$6:N$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",N$6:N$37)+SUMIF($B$6:$B$37,"Delinquency",N$6:N$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",N$6:N$37)+SUMIF($B$6:$B$37,"Other Income",N$6:N$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",N$6:N$37)</f>
+        <f>IF(COUNTIF($B$6:$B$37,"Gross Scheduled Rent")&gt;0,SUMIF($B$6:$B$37,"Gross Scheduled Rent",N$6:N$37),SUMIF($B$6:$B$37,"Gross Potential Rent",N$6:N$37)+SUMIF($B$6:$B$37,"Gain/(Loss) to Lease",N$6:N$37))+SUMIF($B$6:$B$37,"Vacancy",N$6:N$37)+SUMIF($B$6:$B$37,"Concessions",N$6:N$37)+SUMIF($B$6:$B$37,"Non-Revenue Units",N$6:N$37)+SUMIF($B$6:$B$37,"Delinquency",N$6:N$37)+SUMIF($B$6:$B$37,"Utility Reimbursements",N$6:N$37)+SUMIF($B$6:$B$37,"Other Income",N$6:N$37)+SUMIF($B$6:$B$37,"Revenue Adjustments",N$6:N$37)</f>
         <v/>
       </c>
       <c r="O39" s="11">

</xml_diff>

<commit_message>
restage the fixture: case-insensitive categories and a cap-accurate narrative
Two small corrections reach the published set. Category normalization is
case-insensitive on the canonical spellings again (Excel's SUMIF is, so 'payroll'
and 'Payroll' genuinely do tie out) - changing the canonicals last round had removed
the lowercase entries that covered this.

And the comp-set narrative names the CONFIGURED cap rather than the size of the set
it produced, so the fixture no longer says "fewer than 11 qualify either way" when
the cap is 20.
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-t12-analysis.xlsx
+++ b/public/downloads/underwriting-demo/sample-t12-analysis.xlsx
@@ -3475,7 +3475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -3871,115 +3871,107 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Occupied units</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="n">
-        <v>177</v>
-      </c>
+          <t>Duplicate rows: kept the in-place lease</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="n"/>
       <c r="C23" s="17" t="n"/>
       <c r="D23" s="17" t="n"/>
       <c r="E23" s="5" t="inlineStr">
         <is>
+          <t>NOT CHECKED</t>
+        </is>
+      </c>
+      <c r="F23" s="18" t="inlineStr">
+        <is>
+          <t>The export lists no unit twice, so there is no row choice to make.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Occupied units</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>177</v>
+      </c>
+      <c r="C24" s="17" t="n"/>
+      <c r="D24" s="17" t="n"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F23" s="18" t="inlineStr">
+      <c r="F24" s="18" t="inlineStr">
         <is>
           <t>The numerator above, stated separately so the ratio can be re-derived.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>1/5 tie-outs OK; 3 NOT CHECKED</t>
-        </is>
-      </c>
-    </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>1/6 tie-outs OK; 4 NOT CHECKED</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>A total the source export never printed reads NOT CHECKED and stays in the denominator above — excluding it would let a check that could not run flatter the ratio. Occupancy here is PHYSICAL: 177/180 units, physical. Down, model and employee units count as vacant.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>Rent readback — 10 units, sampled reproducibly</t>
         </is>
       </c>
-      <c r="B28" s="16" t="n"/>
-      <c r="C28" s="16" t="n"/>
-      <c r="D28" s="16" t="n"/>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="16" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="B29" s="16" t="n"/>
+      <c r="C29" s="16" t="n"/>
+      <c r="D29" s="16" t="n"/>
+      <c r="E29" s="16" t="n"/>
+      <c r="F29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>Plan</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Our in-place rent</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Source cell value</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Source locator</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>A1-123</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="n">
-        <v>1417</v>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>1417</v>
-      </c>
-      <c r="E30" s="5" t="inlineStr">
-        <is>
-          <t>Rent Roll (source)!F26</t>
-        </is>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>A1-130</t>
+          <t>A1-123</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
@@ -3988,14 +3980,14 @@
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>1438</v>
+        <v>1417</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>1438</v>
+        <v>1417</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll (source)!F33</t>
+          <t>Rent Roll (source)!F26</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -4007,23 +3999,23 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>A2-108</t>
+          <t>A1-130</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>A1</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>1564</v>
+        <v>1438</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>1564</v>
+        <v>1438</v>
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll (source)!F45</t>
+          <t>Rent Roll (source)!F33</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -4035,23 +4027,23 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>B1-101</t>
+          <t>A2-108</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>A2</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>1831</v>
+        <v>1564</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>1831</v>
+        <v>1564</v>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll (source)!F66</t>
+          <t>Rent Roll (source)!F45</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -4063,7 +4055,7 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>B1-103</t>
+          <t>B1-101</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
@@ -4072,14 +4064,14 @@
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>1809</v>
+        <v>1831</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>1809</v>
+        <v>1831</v>
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll (source)!F68</t>
+          <t>Rent Roll (source)!F66</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -4091,7 +4083,7 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>B1-113</t>
+          <t>B1-103</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
@@ -4100,14 +4092,14 @@
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>1734</v>
+        <v>1809</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>1734</v>
+        <v>1809</v>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll (source)!F78</t>
+          <t>Rent Roll (source)!F68</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
@@ -4119,7 +4111,7 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>B1-126</t>
+          <t>B1-113</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
@@ -4128,14 +4120,14 @@
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>1799</v>
+        <v>1734</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>1799</v>
+        <v>1734</v>
       </c>
       <c r="E36" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll (source)!F91</t>
+          <t>Rent Roll (source)!F78</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
@@ -4147,23 +4139,23 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>B2-123</t>
+          <t>B1-126</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>1887</v>
+        <v>1799</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>1887</v>
+        <v>1799</v>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll (source)!F130</t>
+          <t>Rent Roll (source)!F91</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
@@ -4175,23 +4167,23 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>C1-118</t>
+          <t>B2-123</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
-        <v>2056</v>
+        <v>1887</v>
       </c>
       <c r="D38" s="6" t="n">
-        <v>2056</v>
+        <v>1887</v>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Rent Roll (source)!F161</t>
+          <t>Rent Roll (source)!F130</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
@@ -4203,288 +4195,316 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
+          <t>C1-118</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="n">
+        <v>2056</v>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>2056</v>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Rent Roll (source)!F161</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
           <t>Cypress-106</t>
         </is>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>Cypress TH</t>
         </is>
       </c>
-      <c r="C39" s="6" t="n">
+      <c r="C40" s="6" t="n">
         <v>2343</v>
       </c>
-      <c r="D39" s="6" t="n">
+      <c r="D40" s="6" t="n">
         <v>2343</v>
       </c>
-      <c r="E39" s="5" t="inlineStr">
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>Rent Roll (source)!F175</t>
         </is>
       </c>
-      <c r="F39" s="5" t="inlineStr">
+      <c r="F40" s="5" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>10 of 10 match within $0.50. Sample seeded from the roll's as-of date (2026-06-30|180), so the same roll always checks the same units and a reviewer re-running this sees these rows.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="34" customHeight="1">
-      <c r="A42" s="20" t="inlineStr">
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="20" t="inlineStr">
         <is>
           <t>Both sides of the readback read the same rent column, so it validates TRANSCRIPTION — that the number was carried across correctly — and cannot detect the wrong column having been chosen in the first place. The column choice is evidenced in the audit trail instead.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="16" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>Pricing and cap rate (illustrative)</t>
         </is>
       </c>
-      <c r="B44" s="16" t="n"/>
-      <c r="C44" s="16" t="n"/>
-      <c r="D44" s="16" t="n"/>
-      <c r="E44" s="16" t="n"/>
-      <c r="F44" s="16" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Price per unit</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="n">
-        <v>215000</v>
-      </c>
-      <c r="C45" s="20" t="inlineStr">
-        <is>
-          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen to sit inside the band a real per-unit sale price occupies; it is not a quote, an offer, or a broker's guidance.</t>
-        </is>
-      </c>
+      <c r="B45" s="16" t="n"/>
+      <c r="C45" s="16" t="n"/>
+      <c r="D45" s="16" t="n"/>
+      <c r="E45" s="16" t="n"/>
+      <c r="F45" s="16" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Unit count</t>
+          <t>Price per unit</t>
         </is>
       </c>
       <c r="B46" s="6" t="n">
-        <v>180</v>
+        <v>215000</v>
+      </c>
+      <c r="C46" s="20" t="inlineStr">
+        <is>
+          <t>Every price and cap rate below is illustrative. The per-unit price is a round number chosen to sit inside the band a real per-unit sale price occupies; it is not a quote, an offer, or a broker's guidance.</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
+          <t>Unit count</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
           <t>Total purchase price</t>
         </is>
       </c>
-      <c r="B47" s="6">
-        <f>B45*B46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>T-12 revenue</t>
-        </is>
-      </c>
-      <c r="B49" s="6">
-        <f>'P&amp;L Summary'!B16</f>
+      <c r="B48" s="6">
+        <f>B46*B47</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>T-12 operating expenses</t>
+          <t>T-12 revenue</t>
         </is>
       </c>
       <c r="B50" s="6">
-        <f>'P&amp;L Summary'!B29</f>
+        <f>'P&amp;L Summary'!B16</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>T-12 net operating income</t>
+          <t>T-12 operating expenses</t>
         </is>
       </c>
       <c r="B51" s="6">
-        <f>'P&amp;L Summary'!B30</f>
+        <f>'P&amp;L Summary'!B29</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
+          <t>T-12 net operating income</t>
+        </is>
+      </c>
+      <c r="B52" s="6">
+        <f>'P&amp;L Summary'!B30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
           <t>T-12 cap rate (illustrative)</t>
         </is>
       </c>
-      <c r="B52" s="21">
-        <f>IFERROR(B51/B47,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>T-3 annualized revenue</t>
-        </is>
-      </c>
-      <c r="B54" s="6">
-        <f>'P&amp;L Summary'!C16</f>
+      <c r="B53" s="21">
+        <f>IFERROR(B52/B48,"")</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>T-3 annualized operating expenses</t>
+          <t>T-3 annualized revenue</t>
         </is>
       </c>
       <c r="B55" s="6">
-        <f>'P&amp;L Summary'!C29</f>
+        <f>'P&amp;L Summary'!C16</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>T-3 annualized net operating income</t>
+          <t>T-3 annualized operating expenses</t>
         </is>
       </c>
       <c r="B56" s="6">
-        <f>'P&amp;L Summary'!C30</f>
+        <f>'P&amp;L Summary'!C29</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
+          <t>T-3 annualized net operating income</t>
+        </is>
+      </c>
+      <c r="B57" s="6">
+        <f>'P&amp;L Summary'!C30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
           <t>T-3 annualized cap rate (illustrative)</t>
         </is>
       </c>
-      <c r="B57" s="21">
-        <f>IFERROR(B56/B47,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>Broker pro forma revenue</t>
-        </is>
-      </c>
-      <c r="B59" s="6" t="n">
-        <v>4051427.88</v>
-      </c>
-      <c r="C59" s="20" t="inlineStr">
-        <is>
-          <t>Kept in its own block; never merged into the T-12.</t>
-        </is>
+      <c r="B58" s="21">
+        <f>IFERROR(B57/B48,"")</f>
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Broker pro forma operating expenses</t>
+          <t>Broker pro forma revenue</t>
         </is>
       </c>
       <c r="B60" s="6" t="n">
-        <v>1718834.16</v>
+        <v>4051427.88</v>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>Kept in its own block; never merged into the T-12.</t>
+        </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Broker pro forma net operating income</t>
+          <t>Broker pro forma operating expenses</t>
         </is>
       </c>
       <c r="B61" s="6" t="n">
-        <v>2332593.72</v>
+        <v>1718834.16</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
+          <t>Broker pro forma net operating income</t>
+        </is>
+      </c>
+      <c r="B62" s="6" t="n">
+        <v>2332593.72</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
           <t>Broker pro forma cap rate (illustrative)</t>
         </is>
       </c>
-      <c r="B62" s="21">
-        <f>IFERROR(B61/B47,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="16" t="inlineStr">
+      <c r="B63" s="21">
+        <f>IFERROR(B62/B48,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="16" t="inlineStr">
         <is>
           <t>Revenue trend</t>
         </is>
       </c>
-      <c r="B64" s="16" t="n"/>
-      <c r="C64" s="16" t="n"/>
-      <c r="D64" s="16" t="n"/>
-      <c r="E64" s="16" t="n"/>
-      <c r="F64" s="16" t="n"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="5" t="inlineStr">
-        <is>
-          <t>T-12 revenue</t>
-        </is>
-      </c>
-      <c r="B65" s="6">
-        <f>'P&amp;L Summary'!B16</f>
-        <v/>
-      </c>
+      <c r="B65" s="16" t="n"/>
+      <c r="C65" s="16" t="n"/>
+      <c r="D65" s="16" t="n"/>
+      <c r="E65" s="16" t="n"/>
+      <c r="F65" s="16" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>T-6 revenue (annualized)</t>
+          <t>T-12 revenue</t>
         </is>
       </c>
       <c r="B66" s="6">
-        <f>SUM('T-12 Data'!I39:N39)*2</f>
-        <v/>
-      </c>
-      <c r="C66" s="20" t="inlineStr">
-        <is>
-          <t>Trailing six months times two, off the T-12 Data tab's computed revenue row.</t>
-        </is>
+        <f>'P&amp;L Summary'!B16</f>
+        <v/>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>T-3 revenue (annualized)</t>
+          <t>T-6 revenue (annualized)</t>
         </is>
       </c>
       <c r="B67" s="6">
-        <f>'P&amp;L Summary'!C16</f>
-        <v/>
+        <f>SUM('T-12 Data'!I39:N39)*2</f>
+        <v/>
+      </c>
+      <c r="C67" s="20" t="inlineStr">
+        <is>
+          <t>Trailing six months times two, off the T-12 Data tab's computed revenue row.</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
+          <t>T-3 revenue (annualized)</t>
+        </is>
+      </c>
+      <c r="B68" s="6">
+        <f>'P&amp;L Summary'!C16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
           <t>T-3 versus T-12</t>
         </is>
       </c>
-      <c r="B68" s="19">
-        <f>IFERROR(B67/B49-1,"")</f>
-        <v/>
-      </c>
-      <c r="C68" s="20" t="inlineStr">
+      <c r="B69" s="19">
+        <f>IFERROR(B68/B50-1,"")</f>
+        <v/>
+      </c>
+      <c r="C69" s="20" t="inlineStr">
         <is>
           <t>Positive means the trailing three months are running ahead of the year.</t>
         </is>

</xml_diff>

<commit_message>
restage the fixture: cap-consistent narrative and market-rent tie-out inputs
The comp-set note stated two different cap numbers on the fixture ("closest-11" and
"fewer than 20"); it now uses the configured cap throughout. And fixture units carry
a market rent so the completeness tie-out actually runs there - without it the check
reported NOT CHECKED and a test depending on its verdict could not tell "ran and
passed" from "never ran".
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-t12-analysis.xlsx
+++ b/public/downloads/underwriting-demo/sample-t12-analysis.xlsx
@@ -3854,17 +3854,23 @@
           <t>Market rent (monthly total)</t>
         </is>
       </c>
-      <c r="B22" s="17" t="n"/>
-      <c r="C22" s="17" t="n"/>
-      <c r="D22" s="17" t="n"/>
+      <c r="B22" s="6" t="n">
+        <v>342300.5</v>
+      </c>
+      <c r="C22" s="6" t="n">
+        <v>342300.5</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t>NOT CHECKED</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>The parse did not capture a per-unit market rent, so this cannot be tied.</t>
+          <t>Validates row COMPLETENESS — 180 units counted once each, none dropped or double-counted. It does NOT validate which row was kept on a duplicate: all 3 turnover pair(s) here carry the same market rent on both rows, so this total is identical under either de-duplication rule while in-place rent is not. The row CHOICE is checked separately below.</t>
         </is>
       </c>
     </row>
@@ -3874,17 +3880,23 @@
           <t>Duplicate rows: kept the in-place lease</t>
         </is>
       </c>
-      <c r="B23" s="17" t="n"/>
-      <c r="C23" s="17" t="n"/>
-      <c r="D23" s="17" t="n"/>
+      <c r="B23" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>NOT CHECKED</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
-          <t>The export lists no unit twice, so there is no row choice to make.</t>
+          <t>3 unit(s) listed twice; every one where an in-place row was available retained it (1 had none — D-NOCUR, where the alternative row carries no status and no rent, so keeping the other is correct). Keeping the other row instead would move in-place rent by $1,599/mo ($19,188/yr) — which the market-rent tie-out above cannot see.</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3925,7 @@
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>1/6 tie-outs OK; 4 NOT CHECKED</t>
+          <t>3/6 tie-outs OK; 2 NOT CHECKED</t>
         </is>
       </c>
     </row>

</xml_diff>